<commit_message>
Add duplicate attendance status to ScanWindow
</commit_message>
<xml_diff>
--- a/Sessions/2nd October session 12.xlsx
+++ b/Sessions/2nd October session 12.xlsx
@@ -560,17 +560,17 @@
           <t>null 2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[02:44:06]</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>[16:29:34]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[16:29:34] Canceled.</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>excel_import</t>

</xml_diff>

<commit_message>
Add initial Excel file for the session on 3rd October with multiple worksheets and styles
</commit_message>
<xml_diff>
--- a/Sessions/2nd October session 12.xlsx
+++ b/Sessions/2nd October session 12.xlsx
@@ -511,19 +511,17 @@
           <t>null 1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[02:44:04]</t>
+          <t>[00:22:05]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[02:44:04] Attended (Didn't do Homework).</t>
+          <t>[02:44:04] Attended (Didn't do Homework).
+[00:22:05] Canceled.
+[02:44:04] Attended (Didn't do Homework).</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -563,12 +561,16 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[16:29:34]</t>
+          <t>[00:22:25]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[16:29:34] Canceled.</t>
+          <t>[16:29:34] Canceled.
+[16:29:34] Canceled.
+[00:22:25] Canceled.
+[16:29:34] Canceled.
+[16:29:34] Canceled.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -613,19 +615,17 @@
           <t>null 3</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[02:44:09]</t>
+          <t>[18:16:41]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[02:44:09] Completed Homework at center.</t>
+          <t>[02:44:09] Completed Homework at center.
+[18:16:41] Canceled.
+[02:44:09] Completed Homework at center.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -662,8 +662,16 @@
           <t>null 4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[18:16:42]</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
@@ -708,8 +716,30 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[00:24:33]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[18:16:50] Denied Entry: No Homework.
+[00:24:20] Denied Entry: No Exam &amp; Homework.
+[18:16:50] Denied Entry: No Homework.
+[00:24:26] Completed Exam &amp; Homework at center.
+[18:16:50] Denied Entry: No Homework.
+[00:24:20] Denied Entry: No Exam &amp; Homework.
+[18:16:50] Denied Entry: No Homework.
+[00:24:33] Canceled.
+[18:16:50] Denied Entry: No Homework.
+[00:24:20] Denied Entry: No Exam &amp; Homework.
+[18:16:50] Denied Entry: No Homework.
+[00:24:26] Completed Exam &amp; Homework at center.
+[18:16:50] Denied Entry: No Homework.
+[00:24:20] Denied Entry: No Exam &amp; Homework.
+[18:16:50] Denied Entry: No Homework.</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -744,8 +774,16 @@
           <t>null 6</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>[18:16:52]</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
@@ -786,8 +824,16 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>[00:19:59]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>[00:19:59] Canceled.</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -876,8 +922,16 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>[00:21:49]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>[00:21:49] Canceled.</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -920,8 +974,16 @@
           <t>null 10</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>[00:20:22]</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
@@ -965,8 +1027,16 @@
           <t>null 11</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>[00:20:25]</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
@@ -1010,8 +1080,16 @@
           <t>null 12</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>[00:24:10]</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
@@ -1055,8 +1133,16 @@
           <t>null 13</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>[00:24:13]</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
@@ -1190,9 +1276,27 @@
           <t>null 16</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>[00:24:49]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[00:24:40] Attended (Didn't do Exam &amp; Homework).
+[00:24:42] Canceled.
+[00:24:40] Attended (Didn't do Exam &amp; Homework).
+[00:24:49] Completed Exam &amp; Homework at center.
+[00:24:40] Attended (Didn't do Exam &amp; Homework).
+[00:24:42] Canceled.
+[00:24:40] Attended (Didn't do Exam &amp; Homework).</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1227,8 +1331,16 @@
           <t>null 17</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>[00:27:57]</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>

</xml_diff>